<commit_message>
Oturum adları + içerikleri güncellendi, program Excel yenilendi
- Oturum 1: Erzincan-Otlukbeli Oturumu (jeolojik miras, traverten, volkanik yapılar)
- Oturum 2: Erzincan-Çağlayan Oturumu (jeomorfoloji, tufa, KAF zonu)
- Oturum 3: Erzincan-Kemaliye Oturumu (tarihi yapılar, kültürel miras)
- Oturum 4: Erzincan Karma Oturum (biyoloji, tıbbi jeoloji, eğitim)
- Sunum sayıları güncellendi (5, 6, 4, 7)
- 3 dilde içerik açıklamaları eklendi
- Program taslak Excel güncellendi

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/program-taslak.xlsx
+++ b/fotolar/program-taslak.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mehme\OneDrive\Desktop\Çalıştay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D1588F-7DC7-4315-BEC9-35DA9F8EB07D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500752E9-459C-4C0F-9CFD-ADF1289F3E95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="71">
   <si>
     <t>Saat</t>
   </si>
@@ -40,12 +40,6 @@
   </si>
   <si>
     <t>08:30 – 09:30</t>
-  </si>
-  <si>
-    <t>09:30 – 10:00</t>
-  </si>
-  <si>
-    <t>10:00 – 10:15</t>
   </si>
   <si>
     <t>☕ Çay / Kahve Arası</t>
@@ -139,16 +133,10 @@
 sırt ve konileri</t>
   </si>
   <si>
-    <t>10:15 – 12:25</t>
-  </si>
-  <si>
     <t>📊 Bilimsel Sunumlar
 (6 sunum)</t>
   </si>
   <si>
-    <t>12:25 – 13:30</t>
-  </si>
-  <si>
     <t>🍽️ Öğle Yemeği
 (Çağlayan Restoran)</t>
   </si>
@@ -157,19 +145,10 @@
 (Ercan Bey)</t>
   </si>
   <si>
-    <t>13:30 – 15:20</t>
-  </si>
-  <si>
     <t>📊 Bilimsel Sunumlar
 (5 sunum)</t>
   </si>
   <si>
-    <t>15:20 – 15:35</t>
-  </si>
-  <si>
-    <t>15:35 – 16:55</t>
-  </si>
-  <si>
     <t>📊 Bilimsel Sunumlar
 (4 sunum)</t>
   </si>
@@ -178,18 +157,6 @@
 terasları</t>
   </si>
   <si>
-    <t>16:55 – 17:10</t>
-  </si>
-  <si>
-    <t>🔬 OTURUM 4 — KARMA OTURUM</t>
-  </si>
-  <si>
-    <t>17:10 – 19:20</t>
-  </si>
-  <si>
-    <t>🪨 SESSION 1 — GEOLOGICAL HERITAGE</t>
-  </si>
-  <si>
     <t>⛰️ Otlukbeli travertine
 ridge and cones</t>
   </si>
@@ -206,9 +173,6 @@
 (Ercan Bey)</t>
   </si>
   <si>
-    <t>🏔️ SESSION 2 — GEOMORPHOLOGY</t>
-  </si>
-  <si>
     <t>📊 Scientific Presentations
 (5 presentations)</t>
   </si>
@@ -217,9 +181,6 @@
 Active and fossil tufa deposits</t>
   </si>
   <si>
-    <t>🏛️ SESSION 3 — CULTURAL HERITAGE</t>
-  </si>
-  <si>
     <t>📊 Scientific Presentations
 (4 presentations)</t>
   </si>
@@ -228,9 +189,6 @@
 terraces</t>
   </si>
   <si>
-    <t>🔬 SESSION 4 — MIXED SESSION</t>
-  </si>
-  <si>
     <t>🍽️ DINNER
 (Çağlayan Restaurant)</t>
   </si>
@@ -253,34 +211,63 @@
     <t>Uluslararası Katılımlı "Erzincan Jeolojik ve Kültürel Miras"  Çalıştay Programı</t>
   </si>
   <si>
-    <t>🪨 OTURUM 1 — JEOLOJİK MİRAS OTURUMU</t>
-  </si>
-  <si>
     <t>12:30 – 13:30</t>
   </si>
   <si>
-    <t>🏔️ OTURUM 2 — JEOMORFOLOJİ OTURUMU</t>
-  </si>
-  <si>
-    <t>🏛️ OTURUM 3 — KÜLTÜREL MİRAS OTURUMU</t>
-  </si>
-  <si>
-    <t>10:15 – 12:00</t>
-  </si>
-  <si>
-    <t>13:30 – 15:00</t>
-  </si>
-  <si>
-    <t>15:00 – 15:15</t>
-  </si>
-  <si>
-    <t>15:15 – 16:15</t>
-  </si>
-  <si>
-    <t>16:15 – 16:30</t>
-  </si>
-  <si>
-    <t>16:30 – 18:00</t>
+    <t>🪨 OTURUM 1 — ERZİNCAN-OTLUKBELİ OTURUMU</t>
+  </si>
+  <si>
+    <t>09:30 – 10:30</t>
+  </si>
+  <si>
+    <t>10:30 – 10:45</t>
+  </si>
+  <si>
+    <t>10:45 – 11:30</t>
+  </si>
+  <si>
+    <t>🏔️ OTURUM 2 — ERZİNCAN-ÇAĞLAYAN OTURUMU</t>
+  </si>
+  <si>
+    <t>13:30 – 15:15</t>
+  </si>
+  <si>
+    <t>15:15 – 15:30</t>
+  </si>
+  <si>
+    <t>🏛️ OTURUM 3 — ERZİNCAN-KEMALİYE OTURUMU</t>
+  </si>
+  <si>
+    <t>15:30 – 16:30</t>
+  </si>
+  <si>
+    <t>16:30 – 16:45</t>
+  </si>
+  <si>
+    <t>🔬 OTURUM 4 — ERZİNCAN KARMA OTURUM</t>
+  </si>
+  <si>
+    <t>16:45 – 18:30</t>
+  </si>
+  <si>
+    <t>📊 Bilimsel Sunumlar
+(7 sunum)</t>
+  </si>
+  <si>
+    <t>🪨 SESSION 1 — ERZİNCAN-OTLUKBELİ SESSION</t>
+  </si>
+  <si>
+    <t>🏔️ SESSION 2 — ERZİNCAN-ÇAĞLAYAN SESSION</t>
+  </si>
+  <si>
+    <t>🏛️ SESSION 3 — ERZİNCAN-KEMALİYE SESSION</t>
+  </si>
+  <si>
+    <t>🔬 SESSION 4 — ERZİNCAN MIXED SESSION</t>
+  </si>
+  <si>
+    <t>📊 Scientific Presentations
+(7 presentations)</t>
   </si>
 </sst>
 </file>
@@ -677,8 +664,50 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -686,28 +715,16 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -716,57 +733,27 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1047,7 +1034,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="525" row="2">
+  <wetp:taskpane dockstate="right" visibility="0" width="1007" row="2">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1059,9 +1046,7 @@
   <we:alternateReferences>
     <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
   </we:alternateReferences>
-  <we:properties>
-    <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
-  </we:properties>
+  <we:properties/>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </we:webextension>
@@ -1078,28 +1063,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="58" t="s">
-        <v>65</v>
-      </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
+      <c r="A1" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
     </row>
     <row r="2" spans="1:6" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="52" t="s">
+      <c r="B3" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="53"/>
-      <c r="D3" s="52" t="s">
+      <c r="C3" s="39"/>
+      <c r="D3" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="53"/>
+      <c r="E3" s="39"/>
       <c r="F3" s="3" t="s">
         <v>3</v>
       </c>
@@ -1108,194 +1093,194 @@
       <c r="A4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="59" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="39"/>
+      <c r="B4" s="40" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="41"/>
+      <c r="D4" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="43"/>
       <c r="F4" s="4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="56" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="57"/>
-      <c r="D5" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="31"/>
+        <v>54</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="32"/>
+      <c r="D5" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="45"/>
       <c r="F5" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="48" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="49"/>
-      <c r="D6" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="36"/>
+      <c r="D6" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="41"/>
+      <c r="F6" s="5" t="s">
         <v>25</v>
-      </c>
-      <c r="E6" s="60"/>
-      <c r="F6" s="5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="20"/>
-      <c r="B7" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="39"/>
-      <c r="D7" s="56" t="s">
-        <v>32</v>
-      </c>
-      <c r="E7" s="57"/>
+      <c r="B7" s="42" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="43"/>
+      <c r="D7" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="32"/>
       <c r="F7" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="59" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="60"/>
-      <c r="D8" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="E8" s="31"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="45"/>
       <c r="F8" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="B9" s="54" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="55"/>
-      <c r="D9" s="54" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" s="55"/>
+        <v>52</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="30"/>
+      <c r="D9" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="30"/>
       <c r="F9" s="8" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="20"/>
-      <c r="B10" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" s="39"/>
-      <c r="D10" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="35"/>
+      <c r="B10" s="42" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="43"/>
+      <c r="D10" s="46" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="47"/>
       <c r="F10" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="B11" s="56" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="57"/>
-      <c r="D11" s="56" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" s="57"/>
+        <v>58</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="32"/>
+      <c r="D11" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="32"/>
       <c r="F11" s="6" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="B12" s="48" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="49"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="37"/>
+        <v>59</v>
+      </c>
+      <c r="B12" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="36"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="34"/>
       <c r="F12" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="20"/>
-      <c r="B13" s="38" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="39"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="33"/>
+      <c r="B13" s="42" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="43"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="58"/>
       <c r="F13" s="25"/>
     </row>
     <row r="14" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="B14" s="59" t="s">
-        <v>43</v>
-      </c>
-      <c r="C14" s="60"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="37"/>
+        <v>61</v>
+      </c>
+      <c r="B14" s="40" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="41"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="34"/>
       <c r="F14" s="5" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="B15" s="48" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="49"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="33"/>
+        <v>62</v>
+      </c>
+      <c r="B15" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="36"/>
+      <c r="D15" s="57"/>
+      <c r="E15" s="58"/>
       <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="20"/>
-      <c r="B16" s="38" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" s="39"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="37"/>
+      <c r="B16" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="43"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="34"/>
       <c r="F16" s="13"/>
     </row>
     <row r="17" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="B17" s="56" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="57"/>
+        <v>64</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" s="32"/>
       <c r="D17" s="27"/>
       <c r="E17" s="28"/>
       <c r="F17" s="9"/>
@@ -1310,18 +1295,18 @@
     </row>
     <row r="19" spans="1:6" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" s="44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B19" s="52" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="53"/>
+      <c r="D19" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="53"/>
+      <c r="F19" s="14" t="s">
         <v>19</v>
-      </c>
-      <c r="C19" s="45"/>
-      <c r="D19" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="E19" s="45"/>
-      <c r="F19" s="14" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="4" customHeight="1" x14ac:dyDescent="0.35">
@@ -1341,237 +1326,237 @@
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="50"/>
-      <c r="B22" s="50"/>
-      <c r="C22" s="50"/>
-      <c r="D22" s="50"/>
-      <c r="E22" s="50"/>
-      <c r="F22" s="50"/>
+      <c r="A22" s="54"/>
+      <c r="B22" s="54"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="54"/>
     </row>
     <row r="23" spans="1:6" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="24" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="51" t="s">
-        <v>10</v>
-      </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
+      <c r="A24" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" s="55"/>
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
     </row>
     <row r="25" spans="1:6" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="26" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="39"/>
+      <c r="D26" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="B26" s="52" t="s">
+      <c r="E26" s="39"/>
+      <c r="F26" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="C26" s="53"/>
-      <c r="D26" s="52" t="s">
-        <v>13</v>
-      </c>
-      <c r="E26" s="53"/>
-      <c r="F26" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="46" t="s">
-        <v>30</v>
-      </c>
-      <c r="C27" s="47"/>
-      <c r="D27" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="E27" s="39"/>
+      <c r="B27" s="48" t="s">
+        <v>28</v>
+      </c>
+      <c r="C27" s="49"/>
+      <c r="D27" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="E27" s="43"/>
       <c r="F27" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="18" t="s">
-        <v>5</v>
-      </c>
-      <c r="B28" s="40" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" s="41"/>
-      <c r="D28" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="E28" s="31"/>
+        <v>54</v>
+      </c>
+      <c r="B28" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="C28" s="51"/>
+      <c r="D28" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="E28" s="45"/>
       <c r="F28" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B29" s="48" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="49"/>
-      <c r="D29" s="46" t="s">
-        <v>25</v>
-      </c>
-      <c r="E29" s="47"/>
+        <v>55</v>
+      </c>
+      <c r="B29" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="36"/>
+      <c r="D29" s="48" t="s">
+        <v>23</v>
+      </c>
+      <c r="E29" s="49"/>
       <c r="F29" s="15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="20"/>
-      <c r="B30" s="38" t="s">
-        <v>48</v>
-      </c>
-      <c r="C30" s="39"/>
-      <c r="D30" s="40" t="s">
-        <v>28</v>
-      </c>
-      <c r="E30" s="41"/>
+      <c r="B30" s="42" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="43"/>
+      <c r="D30" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="51"/>
       <c r="F30" s="16" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="B31" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="49"/>
+      <c r="D31" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="47"/>
-      <c r="D31" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="E31" s="31"/>
+      <c r="E31" s="45"/>
       <c r="F31" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" s="54" t="s">
-        <v>16</v>
-      </c>
-      <c r="C32" s="55"/>
-      <c r="D32" s="54" t="s">
-        <v>51</v>
-      </c>
-      <c r="E32" s="55"/>
+        <v>52</v>
+      </c>
+      <c r="B32" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="30"/>
+      <c r="D32" s="29" t="s">
+        <v>40</v>
+      </c>
+      <c r="E32" s="30"/>
       <c r="F32" s="8" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="20"/>
-      <c r="B33" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="C33" s="39"/>
-      <c r="D33" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="E33" s="35"/>
+      <c r="B33" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" s="43"/>
+      <c r="D33" s="46" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="47"/>
       <c r="F33" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="C34" s="41"/>
-      <c r="D34" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="E34" s="41"/>
+      <c r="C34" s="51"/>
+      <c r="D34" s="50" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34" s="51"/>
       <c r="F34" s="16" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="B35" s="48" t="s">
-        <v>15</v>
-      </c>
-      <c r="C35" s="49"/>
-      <c r="D35" s="30" t="s">
-        <v>64</v>
-      </c>
-      <c r="E35" s="31"/>
+        <v>59</v>
+      </c>
+      <c r="B35" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" s="36"/>
+      <c r="D35" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="E35" s="45"/>
       <c r="F35" s="7" t="s">
-        <v>64</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="20"/>
-      <c r="B36" s="38" t="s">
-        <v>56</v>
-      </c>
-      <c r="C36" s="39"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="33"/>
+      <c r="B36" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" s="43"/>
+      <c r="D36" s="57"/>
+      <c r="E36" s="58"/>
       <c r="F36" s="25"/>
     </row>
     <row r="37" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="17" t="s">
-        <v>42</v>
-      </c>
-      <c r="B37" s="46" t="s">
-        <v>57</v>
-      </c>
-      <c r="C37" s="47"/>
-      <c r="D37" s="36"/>
-      <c r="E37" s="37"/>
+        <v>61</v>
+      </c>
+      <c r="B37" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="C37" s="49"/>
+      <c r="D37" s="33"/>
+      <c r="E37" s="34"/>
       <c r="F37" s="15" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="B38" s="48" t="s">
-        <v>15</v>
-      </c>
-      <c r="C38" s="49"/>
-      <c r="D38" s="32"/>
-      <c r="E38" s="33"/>
+        <v>62</v>
+      </c>
+      <c r="B38" s="35" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="36"/>
+      <c r="D38" s="57"/>
+      <c r="E38" s="58"/>
       <c r="F38" s="9"/>
     </row>
     <row r="39" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="20"/>
-      <c r="B39" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="C39" s="39"/>
-      <c r="D39" s="36"/>
-      <c r="E39" s="37"/>
+      <c r="B39" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="C39" s="43"/>
+      <c r="D39" s="33"/>
+      <c r="E39" s="34"/>
       <c r="F39" s="13"/>
     </row>
     <row r="40" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B40" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="C40" s="41"/>
-      <c r="D40" s="42"/>
-      <c r="E40" s="43"/>
+        <v>64</v>
+      </c>
+      <c r="B40" s="50" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" s="51"/>
+      <c r="D40" s="59"/>
+      <c r="E40" s="60"/>
       <c r="F40" s="9"/>
     </row>
     <row r="41" spans="1:6" ht="4" customHeight="1" x14ac:dyDescent="0.35">
@@ -1584,18 +1569,18 @@
     </row>
     <row r="42" spans="1:6" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="B42" s="44" t="s">
-        <v>22</v>
-      </c>
-      <c r="C42" s="45"/>
-      <c r="D42" s="44" t="s">
-        <v>60</v>
-      </c>
-      <c r="E42" s="45"/>
+        <v>7</v>
+      </c>
+      <c r="B42" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="C42" s="53"/>
+      <c r="D42" s="52" t="s">
+        <v>46</v>
+      </c>
+      <c r="E42" s="53"/>
       <c r="F42" s="14" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="4" customHeight="1" x14ac:dyDescent="0.35">
@@ -1607,15 +1592,66 @@
       <c r="F43" s="1"/>
     </row>
     <row r="44" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="29"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="29"/>
-      <c r="D44" s="29"/>
-      <c r="E44" s="29"/>
-      <c r="F44" s="29"/>
+      <c r="A44" s="56"/>
+      <c r="B44" s="56"/>
+      <c r="C44" s="56"/>
+      <c r="D44" s="56"/>
+      <c r="E44" s="56"/>
+      <c r="F44" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="67">
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="D14:E14"/>
@@ -1632,57 +1668,6 @@
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Program ve Sunum taslakları güncel halleriyle değiştirildi
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/program-taslak.xlsx
+++ b/fotolar/program-taslak.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mehme\OneDrive\Desktop\Çalıştay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500752E9-459C-4C0F-9CFD-ADF1289F3E95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00995641-FD72-4981-A8B5-83B40E3D2D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5690" yWindow="1400" windowWidth="32710" windowHeight="18040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="69">
   <si>
     <t>Saat</t>
   </si>
@@ -149,10 +149,6 @@
 (5 sunum)</t>
   </si>
   <si>
-    <t>📊 Bilimsel Sunumlar
-(4 sunum)</t>
-  </si>
-  <si>
     <t>🏞️ Güncel traverten
 terasları</t>
   </si>
@@ -181,10 +177,6 @@
 Active and fossil tufa deposits</t>
   </si>
   <si>
-    <t>📊 Scientific Presentations
-(4 presentations)</t>
-  </si>
-  <si>
     <t>🏞️ Active travertine
 terraces</t>
   </si>
@@ -238,36 +230,36 @@
     <t>🏛️ OTURUM 3 — ERZİNCAN-KEMALİYE OTURUMU</t>
   </si>
   <si>
-    <t>15:30 – 16:30</t>
-  </si>
-  <si>
-    <t>16:30 – 16:45</t>
-  </si>
-  <si>
     <t>🔬 OTURUM 4 — ERZİNCAN KARMA OTURUM</t>
   </si>
   <si>
-    <t>16:45 – 18:30</t>
+    <t>🪨 SESSION 1 — ERZİNCAN-OTLUKBELİ SESSION</t>
+  </si>
+  <si>
+    <t>🏔️ SESSION 2 — ERZİNCAN-ÇAĞLAYAN SESSION</t>
+  </si>
+  <si>
+    <t>🏛️ SESSION 3 — ERZİNCAN-KEMALİYE SESSION</t>
+  </si>
+  <si>
+    <t>🔬 SESSION 4 — ERZİNCAN MIXED SESSION</t>
+  </si>
+  <si>
+    <t>15:30 – 16:15</t>
+  </si>
+  <si>
+    <t>16:15 – 16:45</t>
+  </si>
+  <si>
+    <t>16:45 – 18:15</t>
   </si>
   <si>
     <t>📊 Bilimsel Sunumlar
-(7 sunum)</t>
-  </si>
-  <si>
-    <t>🪨 SESSION 1 — ERZİNCAN-OTLUKBELİ SESSION</t>
-  </si>
-  <si>
-    <t>🏔️ SESSION 2 — ERZİNCAN-ÇAĞLAYAN SESSION</t>
-  </si>
-  <si>
-    <t>🏛️ SESSION 3 — ERZİNCAN-KEMALİYE SESSION</t>
-  </si>
-  <si>
-    <t>🔬 SESSION 4 — ERZİNCAN MIXED SESSION</t>
+(3 sunum)</t>
   </si>
   <si>
     <t>📊 Scientific Presentations
-(7 presentations)</t>
+(3 presentations)</t>
   </si>
 </sst>
 </file>
@@ -664,16 +656,25 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -682,78 +683,69 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1034,7 +1026,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="1007" row="2">
+  <wetp:taskpane dockstate="right" visibility="0" width="801" row="2">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1046,7 +1038,9 @@
   <we:alternateReferences>
     <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
   </we:alternateReferences>
-  <we:properties/>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;39fae953-fe9a-4fa6-a1c3-442a146e9a61&quot;"/>
+  </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </we:webextension>
@@ -1063,28 +1057,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="37" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
+      <c r="A1" s="60" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
     </row>
     <row r="2" spans="1:6" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="3" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="39"/>
-      <c r="D3" s="38" t="s">
+      <c r="C3" s="53"/>
+      <c r="D3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="39"/>
+      <c r="E3" s="53"/>
       <c r="F3" s="3" t="s">
         <v>3</v>
       </c>
@@ -1093,194 +1087,194 @@
       <c r="A4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="42" t="s">
+      <c r="C4" s="59"/>
+      <c r="D4" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="43"/>
+      <c r="E4" s="39"/>
       <c r="F4" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="B5" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="32"/>
-      <c r="D5" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="E5" s="45"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="31"/>
       <c r="F5" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="B6" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="36"/>
-      <c r="D6" s="40" t="s">
+      <c r="C6" s="49"/>
+      <c r="D6" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="41"/>
+      <c r="E6" s="59"/>
       <c r="F6" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="20"/>
-      <c r="B7" s="42" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" s="43"/>
-      <c r="D7" s="31" t="s">
+      <c r="B7" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="39"/>
+      <c r="D7" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="32"/>
+      <c r="E7" s="57"/>
       <c r="F7" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="B8" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="41"/>
-      <c r="D8" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="E8" s="45"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="31"/>
       <c r="F8" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="30"/>
-      <c r="D9" s="29" t="s">
+      <c r="C9" s="55"/>
+      <c r="D9" s="54" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="30"/>
+      <c r="E9" s="55"/>
       <c r="F9" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="20"/>
-      <c r="B10" s="42" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="43"/>
-      <c r="D10" s="46" t="s">
-        <v>50</v>
-      </c>
-      <c r="E10" s="47"/>
+      <c r="B10" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="39"/>
+      <c r="D10" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="35"/>
       <c r="F10" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="B11" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="32"/>
-      <c r="D11" s="31" t="s">
+      <c r="C11" s="57"/>
+      <c r="D11" s="56" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="32"/>
+      <c r="E11" s="57"/>
       <c r="F11" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="36"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="34"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="37"/>
       <c r="F12" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="20"/>
-      <c r="B13" s="42" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="43"/>
-      <c r="D13" s="57"/>
-      <c r="E13" s="58"/>
+      <c r="B13" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="39"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="33"/>
       <c r="F13" s="25"/>
     </row>
     <row r="14" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="B14" s="40" t="s">
+        <v>64</v>
+      </c>
+      <c r="B14" s="58" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="59"/>
+      <c r="D14" s="36"/>
+      <c r="E14" s="37"/>
+      <c r="F14" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="C14" s="41"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="58"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="33"/>
       <c r="F15" s="9"/>
     </row>
     <row r="16" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="20"/>
-      <c r="B16" s="42" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="43"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="34"/>
+      <c r="B16" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="39"/>
+      <c r="D16" s="36"/>
+      <c r="E16" s="37"/>
       <c r="F16" s="13"/>
     </row>
     <row r="17" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="B17" s="31" t="s">
-        <v>65</v>
-      </c>
-      <c r="C17" s="32"/>
+        <v>66</v>
+      </c>
+      <c r="B17" s="56" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="57"/>
       <c r="D17" s="27"/>
       <c r="E17" s="28"/>
       <c r="F17" s="9"/>
@@ -1297,14 +1291,14 @@
       <c r="A19" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B19" s="52" t="s">
+      <c r="B19" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="53"/>
-      <c r="D19" s="52" t="s">
+      <c r="C19" s="45"/>
+      <c r="D19" s="44" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="53"/>
+      <c r="E19" s="45"/>
       <c r="F19" s="14" t="s">
         <v>19</v>
       </c>
@@ -1326,37 +1320,37 @@
       <c r="F21" s="1"/>
     </row>
     <row r="22" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="54"/>
-      <c r="B22" s="54"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-      <c r="E22" s="54"/>
-      <c r="F22" s="54"/>
+      <c r="A22" s="50"/>
+      <c r="B22" s="50"/>
+      <c r="C22" s="50"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="50"/>
     </row>
     <row r="23" spans="1:6" ht="10" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="24" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="55" t="s">
+      <c r="A24" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="B24" s="55"/>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="55"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="51"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="51"/>
     </row>
     <row r="25" spans="1:6" ht="6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="26" spans="1:6" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="B26" s="38" t="s">
+      <c r="B26" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="C26" s="39"/>
-      <c r="D26" s="38" t="s">
+      <c r="C26" s="53"/>
+      <c r="D26" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="E26" s="39"/>
+      <c r="E26" s="53"/>
       <c r="F26" s="3" t="s">
         <v>12</v>
       </c>
@@ -1365,198 +1359,198 @@
       <c r="A27" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B27" s="48" t="s">
+      <c r="B27" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C27" s="49"/>
-      <c r="D27" s="42" t="s">
+      <c r="C27" s="47"/>
+      <c r="D27" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="E27" s="43"/>
+      <c r="E27" s="39"/>
       <c r="F27" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="B28" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="51"/>
-      <c r="D28" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="E28" s="45"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="31"/>
       <c r="F28" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="19" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="C29" s="36"/>
-      <c r="D29" s="48" t="s">
+      <c r="C29" s="49"/>
+      <c r="D29" s="46" t="s">
         <v>23</v>
       </c>
-      <c r="E29" s="49"/>
+      <c r="E29" s="47"/>
       <c r="F29" s="15" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="20"/>
-      <c r="B30" s="42" t="s">
-        <v>66</v>
-      </c>
-      <c r="C30" s="43"/>
-      <c r="D30" s="50" t="s">
+      <c r="B30" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="39"/>
+      <c r="D30" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="E30" s="51"/>
+      <c r="E30" s="41"/>
       <c r="F30" s="16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="B31" s="48" t="s">
-        <v>42</v>
-      </c>
-      <c r="C31" s="49"/>
-      <c r="D31" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="E31" s="45"/>
+        <v>54</v>
+      </c>
+      <c r="B31" s="46" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="47"/>
+      <c r="D31" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31" s="31"/>
       <c r="F31" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="B32" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="C32" s="30"/>
-      <c r="D32" s="29" t="s">
+      <c r="C32" s="55"/>
+      <c r="D32" s="54" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" s="55"/>
+      <c r="F32" s="8" t="s">
         <v>40</v>
-      </c>
-      <c r="E32" s="30"/>
-      <c r="F32" s="8" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="20"/>
-      <c r="B33" s="42" t="s">
-        <v>67</v>
-      </c>
-      <c r="C33" s="43"/>
-      <c r="D33" s="46" t="s">
-        <v>50</v>
-      </c>
-      <c r="E33" s="47"/>
+      <c r="B33" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" s="39"/>
+      <c r="D33" s="34" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33" s="35"/>
       <c r="F33" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="18" t="s">
-        <v>58</v>
-      </c>
-      <c r="B34" s="50" t="s">
-        <v>39</v>
-      </c>
-      <c r="C34" s="51"/>
-      <c r="D34" s="50" t="s">
-        <v>43</v>
-      </c>
-      <c r="E34" s="51"/>
+        <v>56</v>
+      </c>
+      <c r="B34" s="40" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" s="41"/>
+      <c r="D34" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="E34" s="41"/>
       <c r="F34" s="16" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="B35" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="C35" s="36"/>
-      <c r="D35" s="44" t="s">
-        <v>50</v>
-      </c>
-      <c r="E35" s="45"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E35" s="31"/>
       <c r="F35" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="20"/>
-      <c r="B36" s="42" t="s">
-        <v>68</v>
-      </c>
-      <c r="C36" s="43"/>
-      <c r="D36" s="57"/>
-      <c r="E36" s="58"/>
+      <c r="B36" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="C36" s="39"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="33"/>
       <c r="F36" s="25"/>
     </row>
     <row r="37" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="17" t="s">
-        <v>61</v>
-      </c>
-      <c r="B37" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="C37" s="49"/>
-      <c r="D37" s="33"/>
-      <c r="E37" s="34"/>
+        <v>64</v>
+      </c>
+      <c r="B37" s="46" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" s="47"/>
+      <c r="D37" s="36"/>
+      <c r="E37" s="37"/>
       <c r="F37" s="15" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B38" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="B38" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="C38" s="36"/>
-      <c r="D38" s="57"/>
-      <c r="E38" s="58"/>
+      <c r="C38" s="49"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="33"/>
       <c r="F38" s="9"/>
     </row>
     <row r="39" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="20"/>
-      <c r="B39" s="42" t="s">
-        <v>69</v>
-      </c>
-      <c r="C39" s="43"/>
-      <c r="D39" s="33"/>
-      <c r="E39" s="34"/>
+      <c r="B39" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" s="39"/>
+      <c r="D39" s="36"/>
+      <c r="E39" s="37"/>
       <c r="F39" s="13"/>
     </row>
     <row r="40" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="B40" s="50" t="s">
-        <v>70</v>
-      </c>
-      <c r="C40" s="51"/>
-      <c r="D40" s="59"/>
-      <c r="E40" s="60"/>
+        <v>66</v>
+      </c>
+      <c r="B40" s="40" t="s">
+        <v>38</v>
+      </c>
+      <c r="C40" s="41"/>
+      <c r="D40" s="42"/>
+      <c r="E40" s="43"/>
       <c r="F40" s="9"/>
     </row>
     <row r="41" spans="1:6" ht="4" customHeight="1" x14ac:dyDescent="0.35">
@@ -1571,16 +1565,16 @@
       <c r="A42" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B42" s="52" t="s">
+      <c r="B42" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="C42" s="53"/>
-      <c r="D42" s="52" t="s">
-        <v>46</v>
-      </c>
-      <c r="E42" s="53"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="E42" s="45"/>
       <c r="F42" s="14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="4" customHeight="1" x14ac:dyDescent="0.35">
@@ -1592,15 +1586,66 @@
       <c r="F43" s="1"/>
     </row>
     <row r="44" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="56"/>
-      <c r="B44" s="56"/>
-      <c r="C44" s="56"/>
-      <c r="D44" s="56"/>
-      <c r="E44" s="56"/>
-      <c r="F44" s="56"/>
+      <c r="A44" s="29"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="29"/>
+      <c r="F44" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="67">
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:E32"/>
     <mergeCell ref="A44:F44"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D31:E31"/>
@@ -1617,57 +1662,6 @@
     <mergeCell ref="D42:E42"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Erzincan Üzümlü Oturum -> Oturumu (TR ekini diğer oturumlarla tutarlı)
Site t4_title + d1_s10_title (statik+i18n TR, 4 yer); program + sunum xlsx
TR başlık hücreleri. EN 'Session' / IT 'Sessione' değişmedi.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/program-taslak.xlsx
+++ b/fotolar/program-taslak.xlsx
@@ -1172,7 +1172,7 @@
       <c r="A16" s="20" t="n"/>
       <c r="B16" s="29" t="inlineStr">
         <is>
-          <t>🔬 OTURUM 4 — ERZİNCAN ÜZÜMLÜ OTURUM</t>
+          <t>🔬 OTURUM 4 — ERZİNCAN ÜZÜMLÜ OTURUMU</t>
         </is>
       </c>
       <c r="C16" s="30" t="n"/>
@@ -1634,8 +1634,8 @@
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="D40:E40"/>
     <mergeCell ref="B27:C27"/>
+    <mergeCell ref="D36:E36"/>
     <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D36:E36"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="D6:E6"/>

</xml_diff>

<commit_message>
Ali Demirsoy Oturum 4'ten Oturum 3 (Kemaliye) basina alindi (roster 5/3/5/3)
- Topics-grid + timeline: Demirsoy O3 (Kemaliye) ilk sira, O4 (Uzumlu)'den cikti
- Sunum sayilari 3 dil: O3 4->5, O4 4->3 (statik + TR/EN/IT i18n)
- Oturum aciklamalari: biyocesitlilik t3_desc'e eklendi, t4_desc'ten cikti (3 dil)
- sunum-taslak.xlsx: O3 5x12dk (14:30-15:30), O4 3x20dk (15:45-16:45)
- program-taslak.xlsx: (5 sunum)/(3 sunum) TR+EN

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/program-taslak.xlsx
+++ b/fotolar/program-taslak.xlsx
@@ -1139,7 +1139,7 @@
       <c r="B14" s="42" t="inlineStr">
         <is>
           <t>📊 Bilimsel Sunumlar
-(4 sunum)</t>
+(5 sunum)</t>
         </is>
       </c>
       <c r="C14" s="30" t="n"/>
@@ -1189,7 +1189,7 @@
       <c r="B17" s="43" t="inlineStr">
         <is>
           <t>📊 Bilimsel Sunumlar
-(4 sunum)</t>
+(3 sunum)</t>
         </is>
       </c>
       <c r="C17" s="30" t="n"/>
@@ -1520,7 +1520,7 @@
       <c r="B37" s="37" t="inlineStr">
         <is>
           <t>📊 Scientific Presentations
-(4 presentations)</t>
+(5 presentations)</t>
         </is>
       </c>
       <c r="C37" s="30" t="n"/>
@@ -1570,7 +1570,7 @@
       <c r="B40" s="34" t="inlineStr">
         <is>
           <t>📊 Scientific Presentations
-(4 presentations)</t>
+(3 presentations)</t>
         </is>
       </c>
       <c r="C40" s="30" t="n"/>
@@ -1633,8 +1633,8 @@
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D36:E36"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D36:E36"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>

</xml_diff>

<commit_message>
1. gun zaman cizelgesi: her oturumda ilk iki sunum 30 dk, kalan 15 dk
- Sunum dosyasi ana kaynak; site + program ona gore senkronlandi
- O2 13:30-14:45, O3 15:00-16:45, O4 17:00-18:15 (ogleden sonrasi kaydi)
- sunum-taslak.xlsx: O2/O3/O4 sunum saatleri 30/30/15 duzenine gore
- program-taslak.xlsx: 1. gun blok saatleri TR+EN yeniden hesaplandi
- index.html: 1. gun timeline blok saatleri (5 blok) guncellendi
- O1 degismedi (Kazanci+Capezzuoli zaten 30'ar dk keynote)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/program-taslak.xlsx
+++ b/fotolar/program-taslak.xlsx
@@ -1070,7 +1070,7 @@
     <row r="11" ht="36" customHeight="1" s="44">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>13:30 – 14:15</t>
+          <t>13:30 – 14:45</t>
         </is>
       </c>
       <c r="B11" s="43" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="12" ht="22" customHeight="1" s="44">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>14:15 – 14:30</t>
+          <t>14:45 – 15:00</t>
         </is>
       </c>
       <c r="B12" s="41" t="inlineStr">
@@ -1133,7 +1133,7 @@
     <row r="14" ht="36" customHeight="1" s="44">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>14:30 – 15:30</t>
+          <t>15:00 – 16:45</t>
         </is>
       </c>
       <c r="B14" s="42" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="15" ht="22" customHeight="1" s="44">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>15:30 – 15:45</t>
+          <t>16:45 – 17:00</t>
         </is>
       </c>
       <c r="B15" s="41" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17" ht="36" customHeight="1" s="44">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>15:45 – 16:45</t>
+          <t>17:00 – 18:15</t>
         </is>
       </c>
       <c r="B17" s="43" t="inlineStr">
@@ -1451,7 +1451,7 @@
     <row r="34" ht="36" customHeight="1" s="44">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>13:30 – 14:15</t>
+          <t>13:30 – 14:45</t>
         </is>
       </c>
       <c r="B34" s="34" t="inlineStr">
@@ -1478,7 +1478,7 @@
     <row r="35" ht="22" customHeight="1" s="44">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>14:15 – 14:30</t>
+          <t>14:45 – 15:00</t>
         </is>
       </c>
       <c r="B35" s="41" t="inlineStr">
@@ -1514,7 +1514,7 @@
     <row r="37" ht="36" customHeight="1" s="44">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>14:30 – 15:30</t>
+          <t>15:00 – 16:45</t>
         </is>
       </c>
       <c r="B37" s="37" t="inlineStr">
@@ -1536,7 +1536,7 @@
     <row r="38" ht="22" customHeight="1" s="44">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>15:30 – 15:45</t>
+          <t>16:45 – 17:00</t>
         </is>
       </c>
       <c r="B38" s="41" t="inlineStr">
@@ -1564,7 +1564,7 @@
     <row r="40" ht="36" customHeight="1" s="44">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>15:45 – 16:45</t>
+          <t>17:00 – 18:15</t>
         </is>
       </c>
       <c r="B40" s="34" t="inlineStr">
@@ -1633,9 +1633,9 @@
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D36:E36"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D36:E36"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="D6:E6"/>

</xml_diff>

<commit_message>
Sunum listesi son hali: kartlara saat+baskan, Inan O1'e (roster 6/3/4/3)
- Calistay Oturumlari kartlari: her sunuma saat onek + blok saati + Oturum Baskanlari (session_chairs i18n 3 dil)
- Kenan Inan O3'ten O1'e tasindi (1473 Otlukbeli); roster 5/3/5/3 -> 6/3/4/3 = 16
- Saatler listeye gore: O1 09:30-11:45, O2 13:30-14:15, O3 14:30-15:30, O4 15:45-16:30 (onceki 30/30/15 iptal)
- Pinar Polat basligi her yerde: 'Konarli Selalesi (Tercan) Ilk Bulgular ve Jeoturizm Potansiyeli'
- Davetli Konusmaci Listesi indirme -> Erjeokum_2026_Sunum_Listesi.xlsx (eski sunum-taslak.xlsx kaldirildi)
- program-taslak.xlsx 1. gun yeni saatlere gore (TR+EN); timeline<->topics birebir senkron

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/program-taslak.xlsx
+++ b/fotolar/program-taslak.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1140" yWindow="1140" windowWidth="32710" windowHeight="18040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5370" yWindow="1320" windowWidth="32710" windowHeight="18040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sayfa1" sheetId="1" state="visible" r:id="rId1"/>
@@ -476,21 +476,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -883,18 +883,18 @@
           <t>Saat</t>
         </is>
       </c>
-      <c r="B3" s="35" t="inlineStr">
+      <c r="B3" s="34" t="inlineStr">
         <is>
           <t>18 Haziran 2026 — Perşembe</t>
         </is>
       </c>
-      <c r="C3" s="36" t="n"/>
-      <c r="D3" s="35" t="inlineStr">
+      <c r="C3" s="35" t="n"/>
+      <c r="D3" s="34" t="inlineStr">
         <is>
           <t>19 Haziran 2026 — Cuma</t>
         </is>
       </c>
-      <c r="E3" s="36" t="n"/>
+      <c r="E3" s="35" t="n"/>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>20 Haziran 2026 — Cumartesi</t>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="C5" s="30" t="n"/>
-      <c r="D5" s="40" t="inlineStr">
+      <c r="D5" s="39" t="inlineStr">
         <is>
           <t>▼</t>
         </is>
@@ -999,17 +999,17 @@
     <row r="8" ht="36" customHeight="1" s="44">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>10:45 – 11:30</t>
+          <t>10:45 – 11:45</t>
         </is>
       </c>
       <c r="B8" s="42" t="inlineStr">
         <is>
           <t>📊 Bilimsel Sunumlar
-(5 sunum)</t>
+(6 sunum)</t>
         </is>
       </c>
       <c r="C8" s="30" t="n"/>
-      <c r="D8" s="40" t="inlineStr">
+      <c r="D8" s="39" t="inlineStr">
         <is>
           <t>▼</t>
         </is>
@@ -1070,7 +1070,7 @@
     <row r="11" ht="36" customHeight="1" s="44">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>13:30 – 14:45</t>
+          <t>13:30 – 14:15</t>
         </is>
       </c>
       <c r="B11" s="43" t="inlineStr">
@@ -1097,7 +1097,7 @@
     <row r="12" ht="22" customHeight="1" s="44">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>14:45 – 15:00</t>
+          <t>14:15 – 14:30</t>
         </is>
       </c>
       <c r="B12" s="41" t="inlineStr">
@@ -1126,20 +1126,20 @@
         </is>
       </c>
       <c r="C13" s="30" t="n"/>
-      <c r="D13" s="39" t="n"/>
+      <c r="D13" s="40" t="n"/>
       <c r="E13" s="30" t="n"/>
       <c r="F13" s="25" t="n"/>
     </row>
     <row r="14" ht="36" customHeight="1" s="44">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>15:00 – 16:45</t>
+          <t>14:30 – 15:30</t>
         </is>
       </c>
       <c r="B14" s="42" t="inlineStr">
         <is>
           <t>📊 Bilimsel Sunumlar
-(5 sunum)</t>
+(4 sunum)</t>
         </is>
       </c>
       <c r="C14" s="30" t="n"/>
@@ -1155,7 +1155,7 @@
     <row r="15" ht="22" customHeight="1" s="44">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>16:45 – 17:00</t>
+          <t>15:30 – 15:45</t>
         </is>
       </c>
       <c r="B15" s="41" t="inlineStr">
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="C15" s="30" t="n"/>
-      <c r="D15" s="39" t="n"/>
+      <c r="D15" s="40" t="n"/>
       <c r="E15" s="30" t="n"/>
       <c r="F15" s="9" t="n"/>
     </row>
@@ -1183,7 +1183,7 @@
     <row r="17" ht="36" customHeight="1" s="44">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>17:00 – 18:15</t>
+          <t>15:45 – 16:30</t>
         </is>
       </c>
       <c r="B17" s="43" t="inlineStr">
@@ -1263,18 +1263,18 @@
           <t>Time</t>
         </is>
       </c>
-      <c r="B26" s="35" t="inlineStr">
+      <c r="B26" s="34" t="inlineStr">
         <is>
           <t>18 June 2026 — Thursday</t>
         </is>
       </c>
-      <c r="C26" s="36" t="n"/>
-      <c r="D26" s="35" t="inlineStr">
+      <c r="C26" s="35" t="n"/>
+      <c r="D26" s="34" t="inlineStr">
         <is>
           <t>19 June 2026 — Friday</t>
         </is>
       </c>
-      <c r="E26" s="36" t="n"/>
+      <c r="E26" s="35" t="n"/>
       <c r="F26" s="3" t="inlineStr">
         <is>
           <t>20 June 2026 — Saturday</t>
@@ -1312,14 +1312,14 @@
           <t>09:30 – 10:00</t>
         </is>
       </c>
-      <c r="B28" s="34" t="inlineStr">
+      <c r="B28" s="36" t="inlineStr">
         <is>
           <t>🎤 Nizamettin Kazancı
 (President of JEMİRKO, Chair of the Natural Sciences Committee, UNESCO Turkey National Committee)</t>
         </is>
       </c>
       <c r="C28" s="30" t="n"/>
-      <c r="D28" s="40" t="inlineStr">
+      <c r="D28" s="39" t="inlineStr">
         <is>
           <t>▼</t>
         </is>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="C30" s="30" t="n"/>
-      <c r="D30" s="34" t="inlineStr">
+      <c r="D30" s="36" t="inlineStr">
         <is>
           <t>🌋 Volcanic cones and
 Altıntepe Mound</t>
@@ -1380,17 +1380,17 @@
     <row r="31" ht="36" customHeight="1" s="44">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>10:45 – 11:30</t>
+          <t>10:45 – 11:45</t>
         </is>
       </c>
       <c r="B31" s="37" t="inlineStr">
         <is>
           <t>📊 Scientific Presentations
-(5 presentations)</t>
+(6 presentations)</t>
         </is>
       </c>
       <c r="C31" s="30" t="n"/>
-      <c r="D31" s="40" t="inlineStr">
+      <c r="D31" s="39" t="inlineStr">
         <is>
           <t>▼</t>
         </is>
@@ -1451,17 +1451,17 @@
     <row r="34" ht="36" customHeight="1" s="44">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>13:30 – 14:45</t>
-        </is>
-      </c>
-      <c r="B34" s="34" t="inlineStr">
+          <t>13:30 – 14:15</t>
+        </is>
+      </c>
+      <c r="B34" s="36" t="inlineStr">
         <is>
           <t>📊 Scientific Presentations
 (3 presentations)</t>
         </is>
       </c>
       <c r="C34" s="30" t="n"/>
-      <c r="D34" s="34" t="inlineStr">
+      <c r="D34" s="36" t="inlineStr">
         <is>
           <t>🌊 Çağlayan &amp; Gürlevik Waterfalls:
 Active and fossil tufa deposits</t>
@@ -1478,7 +1478,7 @@
     <row r="35" ht="22" customHeight="1" s="44">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>14:45 – 15:00</t>
+          <t>14:15 – 14:30</t>
         </is>
       </c>
       <c r="B35" s="41" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="C35" s="30" t="n"/>
-      <c r="D35" s="40" t="inlineStr">
+      <c r="D35" s="39" t="inlineStr">
         <is>
           <t>▼</t>
         </is>
@@ -1507,20 +1507,20 @@
         </is>
       </c>
       <c r="C36" s="30" t="n"/>
-      <c r="D36" s="39" t="n"/>
+      <c r="D36" s="40" t="n"/>
       <c r="E36" s="30" t="n"/>
       <c r="F36" s="25" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1" s="44">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>15:00 – 16:45</t>
+          <t>14:30 – 15:30</t>
         </is>
       </c>
       <c r="B37" s="37" t="inlineStr">
         <is>
           <t>📊 Scientific Presentations
-(5 presentations)</t>
+(4 presentations)</t>
         </is>
       </c>
       <c r="C37" s="30" t="n"/>
@@ -1536,7 +1536,7 @@
     <row r="38" ht="22" customHeight="1" s="44">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>16:45 – 17:00</t>
+          <t>15:30 – 15:45</t>
         </is>
       </c>
       <c r="B38" s="41" t="inlineStr">
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="C38" s="30" t="n"/>
-      <c r="D38" s="39" t="n"/>
+      <c r="D38" s="40" t="n"/>
       <c r="E38" s="30" t="n"/>
       <c r="F38" s="9" t="n"/>
     </row>
@@ -1564,10 +1564,10 @@
     <row r="40" ht="36" customHeight="1" s="44">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>17:00 – 18:15</t>
-        </is>
-      </c>
-      <c r="B40" s="34" t="inlineStr">
+          <t>15:45 – 16:30</t>
+        </is>
+      </c>
+      <c r="B40" s="36" t="inlineStr">
         <is>
           <t>📊 Scientific Presentations
 (3 presentations)</t>
@@ -1629,13 +1629,13 @@
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D34:E34"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D34:E34"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D36:E36"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D36:E36"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="D6:E6"/>
@@ -1665,8 +1665,8 @@
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
     <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D9:E9"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D39:E39"/>
     <mergeCell ref="A24:F24"/>
@@ -1674,15 +1674,15 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D42:E42"/>
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="D15:E15"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="D5:E5"/>
     <mergeCell ref="D33:E33"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D29:E29"/>
     <mergeCell ref="D38:E38"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="B36:C36"/>

</xml_diff>

<commit_message>
O3'te Demirsoy ve Atabey 30 dk'ya cikarildi, sonraki saatler kaydirildi
- O3: Demirsoy 14:30-15:00 (30), Atabey 15:00-15:30 (30), V.Gungor 15:30-15:45 (15), Akpinar-Orhan 15:45-16:00 (15) -> O3 14:30-16:00
- cay 16:00-16:15; O4 16:15-17:00 (Tukel/Polat/Seven 15'er)
- O1/O2 degismedi; gala 20:00
- site (topics kartlari + timeline) + Erjeokum_2026_Sunum_Listesi.xlsx + Program Listesi.xlsx (TR+EN) senkron

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fotolar/program-taslak.xlsx
+++ b/fotolar/program-taslak.xlsx
@@ -1133,7 +1133,7 @@
     <row r="14" ht="36" customHeight="1" s="44">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>14:30 – 15:30</t>
+          <t>14:30 – 16:00</t>
         </is>
       </c>
       <c r="B14" s="42" t="inlineStr">
@@ -1155,7 +1155,7 @@
     <row r="15" ht="22" customHeight="1" s="44">
       <c r="A15" s="19" t="inlineStr">
         <is>
-          <t>15:30 – 15:45</t>
+          <t>16:00 – 16:15</t>
         </is>
       </c>
       <c r="B15" s="41" t="inlineStr">
@@ -1183,7 +1183,7 @@
     <row r="17" ht="36" customHeight="1" s="44">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t>15:45 – 16:30</t>
+          <t>16:15 – 17:00</t>
         </is>
       </c>
       <c r="B17" s="43" t="inlineStr">
@@ -1514,7 +1514,7 @@
     <row r="37" ht="36" customHeight="1" s="44">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>14:30 – 15:30</t>
+          <t>14:30 – 16:00</t>
         </is>
       </c>
       <c r="B37" s="37" t="inlineStr">
@@ -1536,7 +1536,7 @@
     <row r="38" ht="22" customHeight="1" s="44">
       <c r="A38" s="19" t="inlineStr">
         <is>
-          <t>15:30 – 15:45</t>
+          <t>16:00 – 16:15</t>
         </is>
       </c>
       <c r="B38" s="41" t="inlineStr">
@@ -1564,7 +1564,7 @@
     <row r="40" ht="36" customHeight="1" s="44">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>15:45 – 16:30</t>
+          <t>16:15 – 17:00</t>
         </is>
       </c>
       <c r="B40" s="36" t="inlineStr">
@@ -1633,9 +1633,9 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D36:E36"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D36:E36"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="D6:E6"/>

</xml_diff>